<commit_message>
Latest generated outputs 2026-09-23
</commit_message>
<xml_diff>
--- a/generated/spreadsheet/advertising-consent-advertising.xlsx
+++ b/generated/spreadsheet/advertising-consent-advertising.xlsx
@@ -808,7 +808,7 @@
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>List of codelist references that the document covers</t>
+          <t>Planning requirement references identifying the information this document provides. A document may address more than one requirement. These references identify its coverage; they do not establish that the requirements have been satisfied.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2715,7 +2715,7 @@
       <c r="B68" s="2" t="n"/>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Officer name</t>
+          <t>Planning officer name</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr"/>

</xml_diff>